<commit_message>
Up to sgp core classes to clean up
</commit_message>
<xml_diff>
--- a/included/leaguehistory.xlsx
+++ b/included/leaguehistory.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aflyn\repos\Baseball\FantasySgpSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FantBaseball\FantasySgpSystem\included\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDC89CF9-AE26-4CE5-8359-9970099BD13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F706174-6BD4-40FA-848F-270190C92A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4710" windowWidth="29040" windowHeight="15720" xr2:uid="{CDE96B8F-12BE-474E-931C-48604B977C2E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{CDE96B8F-12BE-474E-931C-48604B977C2E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Historical Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Parameters" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="43">
   <si>
     <t>AVERAGE</t>
   </si>
@@ -467,9 +468,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="4" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
@@ -482,6 +480,9 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -490,35 +491,7 @@
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -1127,12 +1100,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA00790-540E-4A47-8DFE-0C5A82FABDCD}">
   <dimension ref="A1:AB77"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="16" max="16" width="9.140625" style="1"/>
+    <col min="16" max="16" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>2023</v>
       </c>
@@ -1151,7 +1124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -1225,7 +1198,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1317,7 +1290,7 @@
         <v>146.71428571428572</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1409,7 +1382,7 @@
         <v>121.28571428571429</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1501,7 +1474,7 @@
         <v>113.42857142857143</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1593,7 +1566,7 @@
         <v>108.71428571428571</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1685,7 +1658,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1777,7 +1750,7 @@
         <v>97.857142857142861</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1869,7 +1842,7 @@
         <v>95.142857142857139</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1961,7 +1934,7 @@
         <v>84.285714285714292</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2053,7 +2026,7 @@
         <v>75.714285714285708</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -2145,7 +2118,7 @@
         <v>69.142857142857139</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2237,7 +2210,7 @@
         <v>56.142857142857146</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -2329,7 +2302,7 @@
         <v>41.142857142857146</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B15">
         <f t="shared" ref="B15:M15" si="4">-1*SLOPE(B4:B13,$A$4:$A$13)</f>
         <v>11.406060606060606</v>
@@ -2379,7 +2352,7 @@
         <v>6.1515151515151514</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B16">
         <f t="shared" ref="B16:G16" si="5">B15/$D$15</f>
         <v>0.79242105263157891</v>
@@ -2429,7 +2402,7 @@
         <v>0.12437201323367233</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2022</v>
       </c>
@@ -2485,7 +2458,7 @@
         <v>92.714285714285708</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="2" t="s">
         <v>2</v>
       </c>
@@ -2574,7 +2547,7 @@
         <v>10.301587301587301</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1</v>
       </c>
@@ -2666,7 +2639,7 @@
         <v>28.089567627925675</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2</v>
       </c>
@@ -2758,7 +2731,7 @@
         <v>96.5</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>3</v>
       </c>
@@ -2850,7 +2823,7 @@
         <v>789.02380952380997</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>4</v>
       </c>
@@ -2892,7 +2865,7 @@
       </c>
       <c r="P22" s="4"/>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>5</v>
       </c>
@@ -2942,7 +2915,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>6</v>
       </c>
@@ -3007,7 +2980,7 @@
         <v>18.377777777777769</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>7</v>
       </c>
@@ -3054,7 +3027,7 @@
         <v>9.2242424242424246</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>8</v>
       </c>
@@ -3146,7 +3119,7 @@
         <v>18.377777777777769</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:28" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>9</v>
       </c>
@@ -3238,7 +3211,7 @@
         <v>6.7887445887445885</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>10</v>
       </c>
@@ -3330,7 +3303,7 @@
         <v>0.11691119460845709</v>
       </c>
     </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>11</v>
       </c>
@@ -3371,7 +3344,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>12</v>
       </c>
@@ -3463,7 +3436,7 @@
         <v>8.0142857142857142</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B31">
         <f t="shared" ref="B31:M31" si="13">-1*SLOPE(B20:B29,$A$20:$A$29)</f>
         <v>10.32121212121212</v>
@@ -3564,7 +3537,7 @@
         <v>9.5974025974025992</v>
       </c>
     </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B32">
         <f t="shared" ref="B32:G32" si="15">B31/$D$31</f>
         <v>0.53858317520556609</v>
@@ -3665,7 +3638,7 @@
         <v>146.71428571428572</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2021</v>
       </c>
@@ -3721,7 +3694,7 @@
         <v>41.142857142857146</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="14" t="s">
         <v>29</v>
       </c>
@@ -3813,7 +3786,7 @@
         <v>30.29691423659164</v>
       </c>
     </row>
-    <row r="35" spans="1:28" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:28" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="14">
         <v>1</v>
       </c>
@@ -3893,7 +3866,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="14">
         <v>2</v>
       </c>
@@ -3970,7 +3943,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="14">
         <v>3</v>
       </c>
@@ -4062,7 +4035,7 @@
         <v>113.42857142857143</v>
       </c>
     </row>
-    <row r="38" spans="1:28" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:28" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="14">
         <v>4</v>
       </c>
@@ -4154,7 +4127,7 @@
         <v>12.603174603174603</v>
       </c>
     </row>
-    <row r="39" spans="1:28" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:28" ht="58.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="14">
         <v>5</v>
       </c>
@@ -4246,7 +4219,7 @@
         <v>116.23203463203461</v>
       </c>
     </row>
-    <row r="40" spans="1:28" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:28" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="14">
         <v>6</v>
       </c>
@@ -4338,7 +4311,7 @@
         <v>12.914670514670512</v>
       </c>
     </row>
-    <row r="41" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="14">
         <v>7</v>
       </c>
@@ -4430,7 +4403,7 @@
         <v>74.071428571428569</v>
       </c>
     </row>
-    <row r="42" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="14">
         <v>8</v>
       </c>
@@ -4522,7 +4495,7 @@
         <v>109.89285714285714</v>
       </c>
     </row>
-    <row r="43" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="14">
         <v>9</v>
       </c>
@@ -4614,7 +4587,7 @@
         <v>35.821428571428569</v>
       </c>
     </row>
-    <row r="44" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="14">
         <v>10</v>
       </c>
@@ -4706,7 +4679,7 @@
         <v>38.25</v>
       </c>
     </row>
-    <row r="45" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="14">
         <v>11</v>
       </c>
@@ -4798,7 +4771,7 @@
         <v>145.71428571428572</v>
       </c>
     </row>
-    <row r="46" spans="1:28" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:28" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="14">
         <v>12</v>
       </c>
@@ -4839,7 +4812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:28" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:28" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B47">
         <f t="shared" ref="B47:G47" si="27">-1*SLOPE(B36:B45,$A$36:$A$45)</f>
         <v>18.145454545454545</v>
@@ -4889,7 +4862,7 @@
         <v>10.036363636363637</v>
       </c>
     </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B48">
         <f t="shared" ref="B48:G48" si="29">B47/$D$47</f>
         <v>1.139269406392694</v>
@@ -4939,564 +4912,564 @@
         <v>0.18769126147568854</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="51" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>2024</v>
       </c>
-      <c r="B51" s="20" t="s">
+      <c r="B51" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20" t="s">
+      <c r="C51" s="24"/>
+      <c r="D51" s="24"/>
+      <c r="E51" s="24"/>
+      <c r="F51" s="24"/>
+      <c r="G51" s="24"/>
+      <c r="H51" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20"/>
-      <c r="L51" s="20"/>
-      <c r="M51" s="20"/>
-    </row>
-    <row r="52" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="21" t="s">
+      <c r="I51" s="24"/>
+      <c r="J51" s="24"/>
+      <c r="K51" s="24"/>
+      <c r="L51" s="24"/>
+      <c r="M51" s="24"/>
+    </row>
+    <row r="52" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B52" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C52" s="21" t="s">
+      <c r="C52" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D52" s="21" t="s">
+      <c r="D52" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="E52" s="21" t="s">
+      <c r="E52" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="F52" s="21" t="s">
+      <c r="F52" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="G52" s="21" t="s">
+      <c r="G52" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="H52" s="21" t="s">
+      <c r="H52" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="I52" s="21" t="s">
+      <c r="I52" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="J52" s="21" t="s">
+      <c r="J52" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="K52" s="21" t="s">
+      <c r="K52" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="L52" s="21" t="s">
+      <c r="L52" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="M52" s="21" t="s">
+      <c r="M52" s="20" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="22">
+    <row r="53" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B53" s="21">
         <v>981</v>
       </c>
-      <c r="C53" s="22">
+      <c r="C53" s="21">
         <v>321</v>
       </c>
-      <c r="D53" s="22">
+      <c r="D53" s="21">
         <v>997</v>
       </c>
-      <c r="E53" s="22">
+      <c r="E53" s="21">
         <v>152</v>
       </c>
-      <c r="F53" s="22">
+      <c r="F53" s="21">
         <v>0.33069999999999999</v>
       </c>
-      <c r="G53" s="22">
+      <c r="G53" s="21">
         <v>0.4577</v>
       </c>
-      <c r="H53" s="22">
+      <c r="H53" s="21">
         <v>1778</v>
       </c>
-      <c r="I53" s="22">
+      <c r="I53" s="21">
         <v>133</v>
       </c>
-      <c r="J53" s="22">
+      <c r="J53" s="21">
         <v>3.4460000000000002</v>
       </c>
-      <c r="K53" s="22">
+      <c r="K53" s="21">
         <v>1.159</v>
       </c>
-      <c r="L53" s="22">
+      <c r="L53" s="21">
         <v>3.4129999999999998</v>
       </c>
-      <c r="M53" s="22">
+      <c r="M53" s="21">
         <v>123</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="23">
+    <row r="54" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B54" s="22">
         <v>1084</v>
       </c>
-      <c r="C54" s="23">
+      <c r="C54" s="22">
         <v>355</v>
       </c>
-      <c r="D54" s="23">
+      <c r="D54" s="22">
         <v>1091</v>
       </c>
-      <c r="E54" s="23">
+      <c r="E54" s="22">
         <v>85</v>
       </c>
-      <c r="F54" s="23">
+      <c r="F54" s="22">
         <v>0.33950000000000002</v>
       </c>
-      <c r="G54" s="23">
+      <c r="G54" s="22">
         <v>0.4476</v>
       </c>
-      <c r="H54" s="23">
+      <c r="H54" s="22">
         <v>1666</v>
       </c>
-      <c r="I54" s="23">
+      <c r="I54" s="22">
         <v>108</v>
       </c>
-      <c r="J54" s="23">
+      <c r="J54" s="22">
         <v>3.621</v>
       </c>
-      <c r="K54" s="23">
+      <c r="K54" s="22">
         <v>1.1499999999999999</v>
       </c>
-      <c r="L54" s="23">
+      <c r="L54" s="22">
         <v>4.1440000000000001</v>
       </c>
-      <c r="M54" s="23">
+      <c r="M54" s="22">
         <v>112</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="22">
+    <row r="55" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B55" s="21">
         <v>969</v>
       </c>
-      <c r="C55" s="22">
+      <c r="C55" s="21">
         <v>279</v>
       </c>
-      <c r="D55" s="22">
+      <c r="D55" s="21">
         <v>941</v>
       </c>
-      <c r="E55" s="22">
+      <c r="E55" s="21">
         <v>111</v>
       </c>
-      <c r="F55" s="22">
+      <c r="F55" s="21">
         <v>0.31969999999999998</v>
       </c>
-      <c r="G55" s="22">
+      <c r="G55" s="21">
         <v>0.4214</v>
       </c>
-      <c r="H55" s="22">
+      <c r="H55" s="21">
         <v>1942</v>
       </c>
-      <c r="I55" s="22">
+      <c r="I55" s="21">
         <v>155</v>
       </c>
-      <c r="J55" s="22">
+      <c r="J55" s="21">
         <v>3.3530000000000002</v>
       </c>
-      <c r="K55" s="22">
+      <c r="K55" s="21">
         <v>1.1399999999999999</v>
       </c>
-      <c r="L55" s="22">
+      <c r="L55" s="21">
         <v>3.6230000000000002</v>
       </c>
-      <c r="M55" s="22">
+      <c r="M55" s="21">
         <v>116</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="22">
+    <row r="56" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B56" s="21">
         <v>1015</v>
       </c>
-      <c r="C56" s="22">
+      <c r="C56" s="21">
         <v>238</v>
       </c>
-      <c r="D56" s="22">
+      <c r="D56" s="21">
         <v>905</v>
       </c>
-      <c r="E56" s="22">
+      <c r="E56" s="21">
         <v>242</v>
       </c>
-      <c r="F56" s="22">
+      <c r="F56" s="21">
         <v>0.314</v>
       </c>
-      <c r="G56" s="22">
+      <c r="G56" s="21">
         <v>0.40739999999999998</v>
       </c>
-      <c r="H56" s="22">
+      <c r="H56" s="21">
         <v>1357</v>
       </c>
-      <c r="I56" s="22">
+      <c r="I56" s="21">
         <v>98</v>
       </c>
-      <c r="J56" s="22">
+      <c r="J56" s="21">
         <v>4.0110000000000001</v>
       </c>
-      <c r="K56" s="22">
+      <c r="K56" s="21">
         <v>1.204</v>
       </c>
-      <c r="L56" s="22">
+      <c r="L56" s="21">
         <v>3.0289999999999999</v>
       </c>
-      <c r="M56" s="22">
+      <c r="M56" s="21">
         <v>115</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="22">
+    <row r="57" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B57" s="21">
         <v>1049</v>
       </c>
-      <c r="C57" s="22">
+      <c r="C57" s="21">
         <v>295</v>
       </c>
-      <c r="D57" s="22">
+      <c r="D57" s="21">
         <v>1007</v>
       </c>
-      <c r="E57" s="22">
+      <c r="E57" s="21">
         <v>177</v>
       </c>
-      <c r="F57" s="22">
+      <c r="F57" s="21">
         <v>0.32640000000000002</v>
       </c>
-      <c r="G57" s="22">
+      <c r="G57" s="21">
         <v>0.43430000000000002</v>
       </c>
-      <c r="H57" s="22">
+      <c r="H57" s="21">
         <v>1419</v>
       </c>
-      <c r="I57" s="22">
+      <c r="I57" s="21">
         <v>83</v>
       </c>
-      <c r="J57" s="22">
+      <c r="J57" s="21">
         <v>4.1109999999999998</v>
       </c>
-      <c r="K57" s="22">
+      <c r="K57" s="21">
         <v>1.2709999999999999</v>
       </c>
-      <c r="L57" s="22">
+      <c r="L57" s="21">
         <v>3.21</v>
       </c>
-      <c r="M57" s="22">
+      <c r="M57" s="21">
         <v>127</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="22">
+    <row r="58" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B58" s="21">
         <v>1065</v>
       </c>
-      <c r="C58" s="22">
+      <c r="C58" s="21">
         <v>249</v>
       </c>
-      <c r="D58" s="22">
+      <c r="D58" s="21">
         <v>975</v>
       </c>
-      <c r="E58" s="22">
+      <c r="E58" s="21">
         <v>250</v>
       </c>
-      <c r="F58" s="22">
+      <c r="F58" s="21">
         <v>0.32369999999999999</v>
       </c>
-      <c r="G58" s="22">
+      <c r="G58" s="21">
         <v>0.4234</v>
       </c>
-      <c r="H58" s="22">
+      <c r="H58" s="21">
         <v>1278</v>
       </c>
-      <c r="I58" s="22">
+      <c r="I58" s="21">
         <v>79</v>
       </c>
-      <c r="J58" s="22">
+      <c r="J58" s="21">
         <v>3.9569999999999999</v>
       </c>
-      <c r="K58" s="22">
+      <c r="K58" s="21">
         <v>1.2689999999999999</v>
       </c>
-      <c r="L58" s="22">
+      <c r="L58" s="21">
         <v>2.766</v>
       </c>
-      <c r="M58" s="22">
+      <c r="M58" s="21">
         <v>87</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="22">
+    <row r="59" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B59" s="21">
         <v>930</v>
       </c>
-      <c r="C59" s="22">
+      <c r="C59" s="21">
         <v>244</v>
       </c>
-      <c r="D59" s="22">
+      <c r="D59" s="21">
         <v>939</v>
       </c>
-      <c r="E59" s="22">
+      <c r="E59" s="21">
         <v>132</v>
       </c>
-      <c r="F59" s="22">
+      <c r="F59" s="21">
         <v>0.31569999999999998</v>
       </c>
-      <c r="G59" s="22">
+      <c r="G59" s="21">
         <v>0.41880000000000001</v>
       </c>
-      <c r="H59" s="22">
+      <c r="H59" s="21">
         <v>1422</v>
       </c>
-      <c r="I59" s="22">
+      <c r="I59" s="21">
         <v>103</v>
       </c>
-      <c r="J59" s="22">
+      <c r="J59" s="21">
         <v>3.6739999999999999</v>
       </c>
-      <c r="K59" s="22">
+      <c r="K59" s="21">
         <v>1.1739999999999999</v>
       </c>
-      <c r="L59" s="22">
+      <c r="L59" s="21">
         <v>3.2170000000000001</v>
       </c>
-      <c r="M59" s="22">
+      <c r="M59" s="21">
         <v>116</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="22">
+    <row r="60" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B60" s="21">
         <v>1070</v>
       </c>
-      <c r="C60" s="22">
+      <c r="C60" s="21">
         <v>295</v>
       </c>
-      <c r="D60" s="22">
+      <c r="D60" s="21">
         <v>985</v>
       </c>
-      <c r="E60" s="22">
+      <c r="E60" s="21">
         <v>193</v>
       </c>
-      <c r="F60" s="22">
+      <c r="F60" s="21">
         <v>0.33350000000000002</v>
       </c>
-      <c r="G60" s="22">
+      <c r="G60" s="21">
         <v>0.43619999999999998</v>
       </c>
-      <c r="H60" s="22">
+      <c r="H60" s="21">
         <v>1598</v>
       </c>
-      <c r="I60" s="22">
+      <c r="I60" s="21">
         <v>113</v>
       </c>
-      <c r="J60" s="22">
+      <c r="J60" s="21">
         <v>4.28</v>
       </c>
-      <c r="K60" s="22">
+      <c r="K60" s="21">
         <v>1.272</v>
       </c>
-      <c r="L60" s="22">
+      <c r="L60" s="21">
         <v>2.9809999999999999</v>
       </c>
-      <c r="M60" s="22">
+      <c r="M60" s="21">
         <v>77</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="22">
+    <row r="61" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B61" s="21">
         <v>976</v>
       </c>
-      <c r="C61" s="22">
+      <c r="C61" s="21">
         <v>285</v>
       </c>
-      <c r="D61" s="22">
+      <c r="D61" s="21">
         <v>951</v>
       </c>
-      <c r="E61" s="22">
+      <c r="E61" s="21">
         <v>134</v>
       </c>
-      <c r="F61" s="22">
+      <c r="F61" s="21">
         <v>0.32329999999999998</v>
       </c>
-      <c r="G61" s="22">
+      <c r="G61" s="21">
         <v>0.44069999999999998</v>
       </c>
-      <c r="H61" s="22">
+      <c r="H61" s="21">
         <v>874</v>
       </c>
-      <c r="I61" s="22">
+      <c r="I61" s="21">
         <v>56</v>
       </c>
-      <c r="J61" s="22">
+      <c r="J61" s="21">
         <v>4.1289999999999996</v>
       </c>
-      <c r="K61" s="22">
+      <c r="K61" s="21">
         <v>1.272</v>
       </c>
-      <c r="L61" s="22">
+      <c r="L61" s="21">
         <v>2.5329999999999999</v>
       </c>
-      <c r="M61" s="22">
+      <c r="M61" s="21">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="22">
+    <row r="62" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B62" s="21">
         <v>908</v>
       </c>
-      <c r="C62" s="22">
+      <c r="C62" s="21">
         <v>203</v>
       </c>
-      <c r="D62" s="22">
+      <c r="D62" s="21">
         <v>889</v>
       </c>
-      <c r="E62" s="22">
+      <c r="E62" s="21">
         <v>158</v>
       </c>
-      <c r="F62" s="22">
+      <c r="F62" s="21">
         <v>0.32969999999999999</v>
       </c>
-      <c r="G62" s="22">
+      <c r="G62" s="21">
         <v>0.4017</v>
       </c>
-      <c r="H62" s="22">
+      <c r="H62" s="21">
         <v>1192</v>
       </c>
-      <c r="I62" s="22">
+      <c r="I62" s="21">
         <v>77</v>
       </c>
-      <c r="J62" s="22">
+      <c r="J62" s="21">
         <v>3.802</v>
       </c>
-      <c r="K62" s="22">
+      <c r="K62" s="21">
         <v>1.133</v>
       </c>
-      <c r="L62" s="22">
+      <c r="L62" s="21">
         <v>3.883</v>
       </c>
-      <c r="M62" s="22">
+      <c r="M62" s="21">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="22">
+    <row r="63" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B63" s="21">
         <v>919</v>
       </c>
-      <c r="C63" s="22">
+      <c r="C63" s="21">
         <v>270</v>
       </c>
-      <c r="D63" s="22">
+      <c r="D63" s="21">
         <v>871</v>
       </c>
-      <c r="E63" s="22">
+      <c r="E63" s="21">
         <v>242</v>
       </c>
-      <c r="F63" s="22">
+      <c r="F63" s="21">
         <v>0.31540000000000001</v>
       </c>
-      <c r="G63" s="22">
+      <c r="G63" s="21">
         <v>0.41739999999999999</v>
       </c>
-      <c r="H63" s="22">
+      <c r="H63" s="21">
         <v>1453</v>
       </c>
-      <c r="I63" s="22">
+      <c r="I63" s="21">
         <v>101</v>
       </c>
-      <c r="J63" s="22">
+      <c r="J63" s="21">
         <v>3.7610000000000001</v>
       </c>
-      <c r="K63" s="22">
+      <c r="K63" s="21">
         <v>1.1779999999999999</v>
       </c>
-      <c r="L63" s="22">
+      <c r="L63" s="21">
         <v>3.34</v>
       </c>
-      <c r="M63" s="22">
+      <c r="M63" s="21">
         <v>93</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="24">
+    <row r="64" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="23">
         <v>907</v>
       </c>
-      <c r="C64" s="24">
+      <c r="C64" s="23">
         <v>251</v>
       </c>
-      <c r="D64" s="24">
+      <c r="D64" s="23">
         <v>846</v>
       </c>
-      <c r="E64" s="24">
+      <c r="E64" s="23">
         <v>125</v>
       </c>
-      <c r="F64" s="24">
+      <c r="F64" s="23">
         <v>0.31359999999999999</v>
       </c>
-      <c r="G64" s="24">
+      <c r="G64" s="23">
         <v>0.41410000000000002</v>
       </c>
-      <c r="H64" s="24">
+      <c r="H64" s="23">
         <v>1231</v>
       </c>
-      <c r="I64" s="24">
+      <c r="I64" s="23">
         <v>70</v>
       </c>
-      <c r="J64" s="24">
+      <c r="J64" s="23">
         <v>3.379</v>
       </c>
-      <c r="K64" s="24">
+      <c r="K64" s="23">
         <v>1.1040000000000001</v>
       </c>
-      <c r="L64" s="24">
+      <c r="L64" s="23">
         <v>3.6419999999999999</v>
       </c>
-      <c r="M64" s="24">
+      <c r="M64" s="23">
         <v>94</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>2024</v>
       </c>
-      <c r="B65" s="21" t="s">
+      <c r="B65" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C65" s="21" t="s">
+      <c r="C65" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D65" s="21" t="s">
+      <c r="D65" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="E65" s="21" t="s">
+      <c r="E65" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="F65" s="21" t="s">
+      <c r="F65" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="G65" s="21" t="s">
+      <c r="G65" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="H65" s="21" t="s">
+      <c r="H65" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="I65" s="21" t="s">
+      <c r="I65" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="J65" s="21" t="s">
+      <c r="J65" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="K65" s="21" t="s">
+      <c r="K65" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="21" t="s">
+      <c r="L65" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="M65" s="21" t="s">
+      <c r="M65" s="20" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B66" cm="1">
         <f t="array" ref="B66:B77">_xlfn._xlws.SORT(B53:B64,,-1)</f>
         <v>1084</v>
@@ -5546,7 +5519,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B67">
         <v>1070</v>
       </c>
@@ -5584,7 +5557,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B68">
         <v>1065</v>
       </c>
@@ -5622,7 +5595,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B69">
         <v>1049</v>
       </c>
@@ -5660,7 +5633,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B70">
         <v>1015</v>
       </c>
@@ -5698,7 +5671,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B71">
         <v>981</v>
       </c>
@@ -5736,7 +5709,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B72">
         <v>976</v>
       </c>
@@ -5774,7 +5747,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B73">
         <v>969</v>
       </c>
@@ -5812,7 +5785,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B74">
         <v>930</v>
       </c>
@@ -5850,7 +5823,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B75">
         <v>919</v>
       </c>
@@ -5888,7 +5861,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B76">
         <v>908</v>
       </c>
@@ -5926,7 +5899,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B77">
         <v>907</v>
       </c>
@@ -5969,31 +5942,181 @@
     <mergeCell ref="B51:G51"/>
     <mergeCell ref="H51:M51"/>
   </mergeCells>
-  <conditionalFormatting sqref="Q3:X14">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="greaterThan">
-      <formula>Q$45</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="lessThan">
+  <conditionalFormatting sqref="Q3:AB14">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>Q$44</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA3:AB14">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
-      <formula>AA$44</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
-      <formula>AA$45</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y3:Z14">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
-      <formula>Y$44</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
-      <formula>Y$45</formula>
+      <formula>Q$45</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9734E317-61B8-40AC-9651-51DC5AB8F31B}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <f>'Historical Data'!$Q26</f>
+        <v>70.609523809523807</v>
+      </c>
+      <c r="C1">
+        <f>'Historical Data'!$Q27</f>
+        <v>15.683982683982686</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <f>'Historical Data'!$R26</f>
+        <v>18.566300366300368</v>
+      </c>
+      <c r="C2">
+        <f>'Historical Data'!$R27</f>
+        <v>7.2874458874458883</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <f>'Historical Data'!$S26</f>
+        <v>67.730402930402946</v>
+      </c>
+      <c r="C3">
+        <f>'Historical Data'!$S27</f>
+        <v>15.613852813852809</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <f>'Historical Data'!$T26</f>
+        <v>7.509743589743592</v>
+      </c>
+      <c r="C4">
+        <f>'Historical Data'!$T27</f>
+        <v>12.555151515151515</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <f>'Historical Data'!$U26</f>
+        <v>0.3165885714285715</v>
+      </c>
+      <c r="C5">
+        <f>'Historical Data'!$U27</f>
+        <v>2.0805194805194839E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <f>'Historical Data'!$V26</f>
+        <v>0.41529809523809524</v>
+      </c>
+      <c r="C6">
+        <f>'Historical Data'!$V27</f>
+        <v>3.3972294372294379E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <f>'Historical Data'!$W26</f>
+        <v>94.228571428571442</v>
+      </c>
+      <c r="C7">
+        <f>'Historical Data'!$W27</f>
+        <v>58.067532467532466</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <f>'Historical Data'!$X26</f>
+        <v>7.663492063492062</v>
+      </c>
+      <c r="C8">
+        <f>'Historical Data'!$X27</f>
+        <v>5.3454545454545466</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <f>'Historical Data'!$Y26</f>
+        <v>4.3037047619047613</v>
+      </c>
+      <c r="C9">
+        <f>'Historical Data'!$Y27</f>
+        <v>-8.6045021645021633E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <f>'Historical Data'!$Z26</f>
+        <v>1.2834761904761904</v>
+      </c>
+      <c r="C10">
+        <f>'Historical Data'!$Z27</f>
+        <v>-1.4143722943722932E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <f>'Historical Data'!$AA26</f>
+        <v>2.7619619047619035</v>
+      </c>
+      <c r="C11">
+        <f>'Historical Data'!$AA27</f>
+        <v>9.4032900432900468E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <f>'Historical Data'!$AB26</f>
+        <v>18.377777777777769</v>
+      </c>
+      <c r="C12">
+        <f>'Historical Data'!$AB27</f>
+        <v>6.7887445887445885</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update to my h2h settings (8SP)
</commit_message>
<xml_diff>
--- a/included/leaguehistory.xlsx
+++ b/included/leaguehistory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aflyn\repos\Baseball\FantasySgpSystem\included\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C6EC73-EF51-4371-A353-82E32C902D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A723A8-34D1-4AF8-888E-3C3069356DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-4695" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CDE96B8F-12BE-474E-931C-48604B977C2E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CDE96B8F-12BE-474E-931C-48604B977C2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Historical Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -513,9 +513,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
@@ -527,6 +524,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3147,8 +3147,8 @@
         <v>92.818181818181827</v>
       </c>
       <c r="X26" s="7">
-        <f>(12*SLOPE(X4:X13,$P$4:$P$13)+INTERCEPT(X4:X13,$P$4:$P$13))/9</f>
-        <v>7.7131313131313117</v>
+        <f>(12*SLOPE(X4:X13,$P$4:$P$13)+INTERCEPT(X4:X13,$P$4:$P$13))/8</f>
+        <v>8.6772727272727259</v>
       </c>
       <c r="Y26" s="7">
         <f>(12*SLOPE(Y4:Y13,$P$4:$P$13)+INTERCEPT(Y4:Y13,$P$4:$P$13))</f>
@@ -3163,8 +3163,8 @@
         <v>2.7432848484848491</v>
       </c>
       <c r="AB26" s="7">
-        <f>(12*SLOPE(AB4:AB13,$P$4:$P$13)+INTERCEPT(AB4:AB13,$P$4:$P$13))/3</f>
-        <v>20.131313131313135</v>
+        <f>(12*SLOPE(AB4:AB13,$P$4:$P$13)+INTERCEPT(AB4:AB13,$P$4:$P$13))/4</f>
+        <v>15.098484848484851</v>
       </c>
     </row>
     <row r="27" spans="1:28" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4965,22 +4965,22 @@
       <c r="A51">
         <v>2024</v>
       </c>
-      <c r="B51" s="24" t="s">
+      <c r="B51" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="C51" s="24"/>
-      <c r="D51" s="24"/>
-      <c r="E51" s="24"/>
-      <c r="F51" s="24"/>
-      <c r="G51" s="24"/>
-      <c r="H51" s="24" t="s">
+      <c r="C51" s="28"/>
+      <c r="D51" s="28"/>
+      <c r="E51" s="28"/>
+      <c r="F51" s="28"/>
+      <c r="G51" s="28"/>
+      <c r="H51" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="I51" s="24"/>
-      <c r="J51" s="24"/>
-      <c r="K51" s="24"/>
-      <c r="L51" s="24"/>
-      <c r="M51" s="24"/>
+      <c r="I51" s="28"/>
+      <c r="J51" s="28"/>
+      <c r="K51" s="28"/>
+      <c r="L51" s="28"/>
+      <c r="M51" s="28"/>
     </row>
     <row r="52" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B52" s="20" t="s">
@@ -6008,496 +6008,496 @@
       <c r="M80" s="29"/>
     </row>
     <row r="81" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B81" s="25" t="s">
+      <c r="B81" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C81" s="25" t="s">
+      <c r="C81" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D81" s="25" t="s">
+      <c r="D81" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E81" s="25" t="s">
+      <c r="E81" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="F81" s="25" t="s">
+      <c r="F81" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="G81" s="25" t="s">
+      <c r="G81" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="H81" s="25" t="s">
+      <c r="H81" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="I81" s="25" t="s">
+      <c r="I81" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="J81" s="25" t="s">
+      <c r="J81" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="K81" s="25" t="s">
+      <c r="K81" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="L81" s="25" t="s">
+      <c r="L81" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="M81" s="25" t="s">
+      <c r="M81" s="24" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="82" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B82" s="26">
+      <c r="B82" s="25">
         <v>1010</v>
       </c>
-      <c r="C82" s="26">
+      <c r="C82" s="25">
         <v>290</v>
       </c>
-      <c r="D82" s="26">
+      <c r="D82" s="25">
         <v>1004</v>
       </c>
-      <c r="E82" s="26">
+      <c r="E82" s="25">
         <v>217</v>
       </c>
-      <c r="F82" s="26">
+      <c r="F82" s="25">
         <v>0.31259999999999999</v>
       </c>
-      <c r="G82" s="26">
+      <c r="G82" s="25">
         <v>0.432</v>
       </c>
-      <c r="H82" s="26">
+      <c r="H82" s="25">
         <v>1627</v>
       </c>
-      <c r="I82" s="26">
+      <c r="I82" s="25">
         <v>105</v>
       </c>
-      <c r="J82" s="26">
+      <c r="J82" s="25">
         <v>3.7679999999999998</v>
       </c>
-      <c r="K82" s="26">
+      <c r="K82" s="25">
         <v>1.222</v>
       </c>
-      <c r="L82" s="26">
+      <c r="L82" s="25">
         <v>2.8439999999999999</v>
       </c>
-      <c r="M82" s="26">
+      <c r="M82" s="25">
         <v>103</v>
       </c>
     </row>
     <row r="83" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="26">
+      <c r="B83" s="25">
         <v>1045</v>
       </c>
-      <c r="C83" s="26">
+      <c r="C83" s="25">
         <v>264</v>
       </c>
-      <c r="D83" s="26">
+      <c r="D83" s="25">
         <v>949</v>
       </c>
-      <c r="E83" s="26">
+      <c r="E83" s="25">
         <v>181</v>
       </c>
-      <c r="F83" s="26">
+      <c r="F83" s="25">
         <v>0.33779999999999999</v>
       </c>
-      <c r="G83" s="26">
+      <c r="G83" s="25">
         <v>0.4325</v>
       </c>
-      <c r="H83" s="26">
+      <c r="H83" s="25">
         <v>1534</v>
       </c>
-      <c r="I83" s="26">
+      <c r="I83" s="25">
         <v>98</v>
       </c>
-      <c r="J83" s="26">
+      <c r="J83" s="25">
         <v>3.7229999999999999</v>
       </c>
-      <c r="K83" s="26">
+      <c r="K83" s="25">
         <v>1.177</v>
       </c>
-      <c r="L83" s="26">
+      <c r="L83" s="25">
         <v>3.306</v>
       </c>
-      <c r="M83" s="26">
+      <c r="M83" s="25">
         <v>114</v>
       </c>
     </row>
     <row r="84" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B84" s="26">
+      <c r="B84" s="25">
         <v>961</v>
       </c>
-      <c r="C84" s="26">
+      <c r="C84" s="25">
         <v>261</v>
       </c>
-      <c r="D84" s="26">
+      <c r="D84" s="25">
         <v>908</v>
       </c>
-      <c r="E84" s="26">
+      <c r="E84" s="25">
         <v>225</v>
       </c>
-      <c r="F84" s="26">
+      <c r="F84" s="25">
         <v>0.32529999999999998</v>
       </c>
-      <c r="G84" s="26">
+      <c r="G84" s="25">
         <v>0.42009999999999997</v>
       </c>
-      <c r="H84" s="26">
+      <c r="H84" s="25">
         <v>1424</v>
       </c>
-      <c r="I84" s="26">
+      <c r="I84" s="25">
         <v>97</v>
       </c>
-      <c r="J84" s="26">
+      <c r="J84" s="25">
         <v>4.141</v>
       </c>
-      <c r="K84" s="26">
+      <c r="K84" s="25">
         <v>1.2450000000000001</v>
       </c>
-      <c r="L84" s="26">
+      <c r="L84" s="25">
         <v>3.1429999999999998</v>
       </c>
-      <c r="M84" s="26">
+      <c r="M84" s="25">
         <v>78</v>
       </c>
     </row>
     <row r="85" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B85" s="26">
+      <c r="B85" s="25">
         <v>1024</v>
       </c>
-      <c r="C85" s="26">
+      <c r="C85" s="25">
         <v>294</v>
       </c>
-      <c r="D85" s="26">
+      <c r="D85" s="25">
         <v>979</v>
       </c>
-      <c r="E85" s="26">
+      <c r="E85" s="25">
         <v>157</v>
       </c>
-      <c r="F85" s="26">
+      <c r="F85" s="25">
         <v>0.34239999999999998</v>
       </c>
-      <c r="G85" s="26">
+      <c r="G85" s="25">
         <v>0.44500000000000001</v>
       </c>
-      <c r="H85" s="26">
+      <c r="H85" s="25">
         <v>1717</v>
       </c>
-      <c r="I85" s="26">
+      <c r="I85" s="25">
         <v>111</v>
       </c>
-      <c r="J85" s="26">
+      <c r="J85" s="25">
         <v>3.7349999999999999</v>
       </c>
-      <c r="K85" s="26">
+      <c r="K85" s="25">
         <v>1.2190000000000001</v>
       </c>
-      <c r="L85" s="26">
+      <c r="L85" s="25">
         <v>2.7559999999999998</v>
       </c>
-      <c r="M85" s="26">
+      <c r="M85" s="25">
         <v>121</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B86" s="26">
+      <c r="B86" s="25">
         <v>1049</v>
       </c>
-      <c r="C86" s="26">
+      <c r="C86" s="25">
         <v>279</v>
       </c>
-      <c r="D86" s="26">
+      <c r="D86" s="25">
         <v>982</v>
       </c>
-      <c r="E86" s="26">
+      <c r="E86" s="25">
         <v>167</v>
       </c>
-      <c r="F86" s="26">
+      <c r="F86" s="25">
         <v>0.32379999999999998</v>
       </c>
-      <c r="G86" s="26">
+      <c r="G86" s="25">
         <v>0.42559999999999998</v>
       </c>
-      <c r="H86" s="26">
+      <c r="H86" s="25">
         <v>1453</v>
       </c>
-      <c r="I86" s="26">
+      <c r="I86" s="25">
         <v>92</v>
       </c>
-      <c r="J86" s="26">
+      <c r="J86" s="25">
         <v>3.6480000000000001</v>
       </c>
-      <c r="K86" s="26">
+      <c r="K86" s="25">
         <v>1.2050000000000001</v>
       </c>
-      <c r="L86" s="26">
+      <c r="L86" s="25">
         <v>2.996</v>
       </c>
-      <c r="M86" s="26">
+      <c r="M86" s="25">
         <v>81</v>
       </c>
     </row>
     <row r="87" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B87" s="27">
+      <c r="B87" s="26">
         <v>1031</v>
       </c>
-      <c r="C87" s="27">
+      <c r="C87" s="26">
         <v>336</v>
       </c>
-      <c r="D87" s="27">
+      <c r="D87" s="26">
         <v>1077</v>
       </c>
-      <c r="E87" s="27">
+      <c r="E87" s="26">
         <v>68</v>
       </c>
-      <c r="F87" s="27">
+      <c r="F87" s="26">
         <v>0.32269999999999999</v>
       </c>
-      <c r="G87" s="27">
+      <c r="G87" s="26">
         <v>0.44169999999999998</v>
       </c>
-      <c r="H87" s="27">
+      <c r="H87" s="26">
         <v>1679</v>
       </c>
-      <c r="I87" s="27">
+      <c r="I87" s="26">
         <v>106</v>
       </c>
-      <c r="J87" s="27">
+      <c r="J87" s="26">
         <v>3.73</v>
       </c>
-      <c r="K87" s="27">
+      <c r="K87" s="26">
         <v>1.2050000000000001</v>
       </c>
-      <c r="L87" s="27">
+      <c r="L87" s="26">
         <v>3.476</v>
       </c>
-      <c r="M87" s="27">
+      <c r="M87" s="26">
         <v>87</v>
       </c>
     </row>
     <row r="88" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B88" s="26">
+      <c r="B88" s="25">
         <v>1008</v>
       </c>
-      <c r="C88" s="26">
+      <c r="C88" s="25">
         <v>290</v>
       </c>
-      <c r="D88" s="26">
+      <c r="D88" s="25">
         <v>944</v>
       </c>
-      <c r="E88" s="26">
+      <c r="E88" s="25">
         <v>121</v>
       </c>
-      <c r="F88" s="26">
+      <c r="F88" s="25">
         <v>0.3266</v>
       </c>
-      <c r="G88" s="26">
+      <c r="G88" s="25">
         <v>0.44090000000000001</v>
       </c>
-      <c r="H88" s="26">
+      <c r="H88" s="25">
         <v>1504</v>
       </c>
-      <c r="I88" s="26">
+      <c r="I88" s="25">
         <v>94</v>
       </c>
-      <c r="J88" s="26">
+      <c r="J88" s="25">
         <v>4.266</v>
       </c>
-      <c r="K88" s="26">
+      <c r="K88" s="25">
         <v>1.2589999999999999</v>
       </c>
-      <c r="L88" s="26">
+      <c r="L88" s="25">
         <v>2.972</v>
       </c>
-      <c r="M88" s="26">
+      <c r="M88" s="25">
         <v>108</v>
       </c>
     </row>
     <row r="89" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B89" s="26">
+      <c r="B89" s="25">
         <v>917</v>
       </c>
-      <c r="C89" s="26">
+      <c r="C89" s="25">
         <v>263</v>
       </c>
-      <c r="D89" s="26">
+      <c r="D89" s="25">
         <v>899</v>
       </c>
-      <c r="E89" s="26">
+      <c r="E89" s="25">
         <v>143</v>
       </c>
-      <c r="F89" s="26">
+      <c r="F89" s="25">
         <v>0.32050000000000001</v>
       </c>
-      <c r="G89" s="26">
+      <c r="G89" s="25">
         <v>0.43090000000000001</v>
       </c>
-      <c r="H89" s="26">
+      <c r="H89" s="25">
         <v>1171</v>
       </c>
-      <c r="I89" s="26">
+      <c r="I89" s="25">
         <v>80</v>
       </c>
-      <c r="J89" s="26">
+      <c r="J89" s="25">
         <v>3.867</v>
       </c>
-      <c r="K89" s="26">
+      <c r="K89" s="25">
         <v>1.2130000000000001</v>
       </c>
-      <c r="L89" s="26">
+      <c r="L89" s="25">
         <v>3.165</v>
       </c>
-      <c r="M89" s="26">
+      <c r="M89" s="25">
         <v>124</v>
       </c>
     </row>
     <row r="90" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="26">
+      <c r="B90" s="25">
         <v>1016</v>
       </c>
-      <c r="C90" s="26">
+      <c r="C90" s="25">
         <v>329</v>
       </c>
-      <c r="D90" s="26">
+      <c r="D90" s="25">
         <v>1029</v>
       </c>
-      <c r="E90" s="26">
+      <c r="E90" s="25">
         <v>193</v>
       </c>
-      <c r="F90" s="26">
+      <c r="F90" s="25">
         <v>0.33189999999999997</v>
       </c>
-      <c r="G90" s="26">
+      <c r="G90" s="25">
         <v>0.46010000000000001</v>
       </c>
-      <c r="H90" s="26">
+      <c r="H90" s="25">
         <v>1148</v>
       </c>
-      <c r="I90" s="26">
+      <c r="I90" s="25">
         <v>63</v>
       </c>
-      <c r="J90" s="26">
+      <c r="J90" s="25">
         <v>3.7029999999999998</v>
       </c>
-      <c r="K90" s="26">
+      <c r="K90" s="25">
         <v>1.228</v>
       </c>
-      <c r="L90" s="26">
+      <c r="L90" s="25">
         <v>3.1030000000000002</v>
       </c>
-      <c r="M90" s="26">
+      <c r="M90" s="25">
         <v>110</v>
       </c>
     </row>
     <row r="91" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B91" s="26">
+      <c r="B91" s="25">
         <v>931</v>
       </c>
-      <c r="C91" s="26">
+      <c r="C91" s="25">
         <v>257</v>
       </c>
-      <c r="D91" s="26">
+      <c r="D91" s="25">
         <v>856</v>
       </c>
-      <c r="E91" s="26">
+      <c r="E91" s="25">
         <v>190</v>
       </c>
-      <c r="F91" s="26">
+      <c r="F91" s="25">
         <v>0.32279999999999998</v>
       </c>
-      <c r="G91" s="26">
+      <c r="G91" s="25">
         <v>0.41070000000000001</v>
       </c>
-      <c r="H91" s="26">
+      <c r="H91" s="25">
         <v>1181</v>
       </c>
-      <c r="I91" s="26">
+      <c r="I91" s="25">
         <v>91</v>
       </c>
-      <c r="J91" s="26">
+      <c r="J91" s="25">
         <v>4.0979999999999999</v>
       </c>
-      <c r="K91" s="26">
+      <c r="K91" s="25">
         <v>1.24</v>
       </c>
-      <c r="L91" s="26">
+      <c r="L91" s="25">
         <v>2.601</v>
       </c>
-      <c r="M91" s="26">
+      <c r="M91" s="25">
         <v>71</v>
       </c>
     </row>
     <row r="92" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B92" s="26">
+      <c r="B92" s="25">
         <v>889</v>
       </c>
-      <c r="C92" s="26">
+      <c r="C92" s="25">
         <v>259</v>
       </c>
-      <c r="D92" s="26">
+      <c r="D92" s="25">
         <v>891</v>
       </c>
-      <c r="E92" s="26">
+      <c r="E92" s="25">
         <v>102</v>
       </c>
-      <c r="F92" s="26">
+      <c r="F92" s="25">
         <v>0.32729999999999998</v>
       </c>
-      <c r="G92" s="26">
+      <c r="G92" s="25">
         <v>0.43070000000000003</v>
       </c>
-      <c r="H92" s="26">
+      <c r="H92" s="25">
         <v>1595</v>
       </c>
-      <c r="I92" s="26">
+      <c r="I92" s="25">
         <v>120</v>
       </c>
-      <c r="J92" s="26">
+      <c r="J92" s="25">
         <v>3.3319999999999999</v>
       </c>
-      <c r="K92" s="26">
+      <c r="K92" s="25">
         <v>1.141</v>
       </c>
-      <c r="L92" s="26">
+      <c r="L92" s="25">
         <v>3.282</v>
       </c>
-      <c r="M92" s="26">
+      <c r="M92" s="25">
         <v>81</v>
       </c>
     </row>
     <row r="93" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="28">
+      <c r="B93" s="27">
         <v>852</v>
       </c>
-      <c r="C93" s="28">
+      <c r="C93" s="27">
         <v>188</v>
       </c>
-      <c r="D93" s="28">
+      <c r="D93" s="27">
         <v>776</v>
       </c>
-      <c r="E93" s="28">
+      <c r="E93" s="27">
         <v>161</v>
       </c>
-      <c r="F93" s="28">
+      <c r="F93" s="27">
         <v>0.32840000000000003</v>
       </c>
-      <c r="G93" s="28">
+      <c r="G93" s="27">
         <v>0.41249999999999998</v>
       </c>
-      <c r="H93" s="28">
+      <c r="H93" s="27">
         <v>963</v>
       </c>
-      <c r="I93" s="28">
+      <c r="I93" s="27">
         <v>43</v>
       </c>
-      <c r="J93" s="28">
+      <c r="J93" s="27">
         <v>3.7429999999999999</v>
       </c>
-      <c r="K93" s="28">
+      <c r="K93" s="27">
         <v>1.175</v>
       </c>
-      <c r="L93" s="28">
+      <c r="L93" s="27">
         <v>3.8210000000000002</v>
       </c>
-      <c r="M93" s="28">
+      <c r="M93" s="27">
         <v>124</v>
       </c>
     </row>
@@ -6505,40 +6505,40 @@
       <c r="A94">
         <v>2025</v>
       </c>
-      <c r="B94" s="25" t="s">
+      <c r="B94" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C94" s="25" t="s">
+      <c r="C94" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D94" s="25" t="s">
+      <c r="D94" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E94" s="25" t="s">
+      <c r="E94" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="F94" s="25" t="s">
+      <c r="F94" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="G94" s="25" t="s">
+      <c r="G94" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="H94" s="25" t="s">
+      <c r="H94" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="I94" s="25" t="s">
+      <c r="I94" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="J94" s="25" t="s">
+      <c r="J94" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="K94" s="25" t="s">
+      <c r="K94" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="L94" s="25" t="s">
+      <c r="L94" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="M94" s="25" t="s">
+      <c r="M94" s="24" t="s">
         <v>13</v>
       </c>
     </row>
@@ -7132,7 +7132,7 @@
       </c>
       <c r="B8">
         <f>'Historical Data'!$X26</f>
-        <v>7.7131313131313117</v>
+        <v>8.6772727272727259</v>
       </c>
       <c r="C8">
         <f>'Historical Data'!$X27</f>
@@ -7184,7 +7184,7 @@
       </c>
       <c r="B12">
         <f>'Historical Data'!$AB26</f>
-        <v>20.131313131313135</v>
+        <v>15.098484848484851</v>
       </c>
       <c r="C12">
         <f>'Historical Data'!$AB27</f>

</xml_diff>